<commit_message>
Replace full product catalog with departments and exception products
A store now needs only a map, a departments sheet (zone + a few example
products) and an optional short list of products shelved outside their
expected department. The LLM assigns each item to a department; RAG
retrieves departments and exceptions. Legacy stores with a full catalog
still load, with departments derived from the catalog categories.

- Ask the user only when the options are in different zones
- Accept an exception product only on a strong name/alias match
  (RAG score >= 0.75); weak models grabbed unrelated candidates
- Accept a bare JSON list from the model for matches and parsed items
- Evals: ground truth is the expected zone per item; scope eval no
  longer counts failed runs as non-refusals
- Rerun evals for the paid models; keep previous results as *_catalog_v1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/store_template.xlsx
+++ b/store_template.xlsx
@@ -9,11 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הוראות" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מפת החנות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מוצרים" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מחלקות" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="חריגים" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'מוצרים'!$A$1:$F$2</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +59,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +94,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -189,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,6 +233,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -598,121 +616,133 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>איך ממלאים את קובץ החנות</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>לשונית 'מפת החנות': מציירים את החנות במבט מלמעלה. כל משבצת היא בערך מטר על מטר.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>לשונית 'מפת החנות': מציירים את החנות במבט מלמעלה. כל משבצת היא בערך מטר על מטר.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    • משבצת ריקה = מקום שאפשר ללכת בו.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • משבצת ריקה = מקום שאפשר ללכת בו.</t>
+          <t xml:space="preserve">    • X = מדף, קיר, מקרר או דלפק. מקום שאי אפשר לעבור דרכו.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • X = מדף, קיר, מקרר או דלפק. מקום שאי אפשר לעבור דרכו.</t>
+          <t xml:space="preserve">    • טקסט (למשל 'מעבר 3', 'חלב וביצים') = המקום שבו הלקוח עומד כשהוא לוקח מוצרים מהאזור.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • טקסט (למשל 'מעבר 3', 'חלב וביצים') = המקום שבו הלקוח עומד כשהוא לוקח מוצרים מהאזור.</t>
+          <t xml:space="preserve">       אפשר לכתוב בתא אחד, או למזג כמה תאים (Merge) ולכתוב בהם פעם אחת.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">       אפשר לכתוב בתא אחד, או למזג כמה תאים (Merge) ולכתוב בהם פעם אחת.</t>
+          <t xml:space="preserve">    • חובה: תא אחד עם המילה 'כניסה' ותא אחד עם המילה 'קופות'.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • חובה: תא אחד עם המילה 'כניסה' ותא אחד עם המילה 'קופות'.</t>
+          <t xml:space="preserve">    • מומלץ להקיף את כל החנות בקיר של X.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • מומלץ להקיף את כל החנות בקיר של X.</t>
+          <t xml:space="preserve">    • שורה 1 היא להגדרות (שם החנות, כמה מטר כל משבצת). את הציור מתחילים משורה 3.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • שורה 1 היא להגדרות (שם החנות, כמה מטר כל משבצת). את הציור מתחילים משורה 3.</t>
+          <t xml:space="preserve">    • צבעים לא חובה. הם רק עוזרים לראות את הציור.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • צבעים לא חובה. הם רק עוזרים לראות את הציור.</t>
+          <t>לשונית 'מחלקות' (חובה): שורה לכל מחלקה.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    • 'אזור' = בדיוק הטקסט שכתבתם בציור (למשל 'מעבר 3'). כמה מחלקות יכולות להיות באותו אזור.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>לשונית 'מוצרים': שורה לכל מוצר.</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    • 'מה נמכר כאן' = כמה דוגמאות מופרדות בפסיקים. לא צריך רשימה מלאה:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • 'אזור' = בדיוק הטקסט שכתבתם בציור (למשל 'מעבר 3').</t>
+          <t xml:space="preserve">       האייג'נט משייך כל מוצר למחלקה המתאימה לפי הדוגמאות ולפי ידע כללי.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • 'שמות נוספים' = איך לקוחות עשויים לכתוב את המוצר, מופרדים ב- |</t>
+          <t>לשונית 'חריגים' (לא חובה): רק מוצרים שלא נמצאים במחלקה שהייתם מצפים לה.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • 'לאסוף בסוף' = 'כן' רק למוצרים שנמסים מהר, כמו גלידה. האזור שלהם יהיה אחרון לפני הקופות.</t>
+          <t xml:space="preserve">    • למשל סוללות ליד הקופות, או חלב סויה במעבר הקפה ולא במקרר החלב.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    • מק"ט וקטגוריה לא חובה.</t>
+          <t xml:space="preserve">    • 'שמות נוספים' = איך לקוחות עשויים לכתוב את המוצר, מופרדים ב- |</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    • 'לאסוף בסוף' = 'כן' למוצר שנמס מהר. (גלידה וארטיק מזוהים גם בלי זה.)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>אם יש טעות (אזור שלא קיים בציור, אזור חסום, חסרה כניסה) המערכת תציג הודעה שמסבירה מה לתקן.</t>
         </is>
@@ -1825,8 +1855,8 @@
           <t>כניסה</t>
         </is>
       </c>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="11" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="24" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
@@ -1852,10 +1882,10 @@
           <t>קופות</t>
         </is>
       </c>
-      <c r="Z26" s="13" t="n"/>
-      <c r="AA26" s="13" t="n"/>
-      <c r="AB26" s="13" t="n"/>
-      <c r="AC26" s="14" t="n"/>
+      <c r="Z26" s="23" t="n"/>
+      <c r="AA26" s="23" t="n"/>
+      <c r="AB26" s="23" t="n"/>
+      <c r="AC26" s="24" t="n"/>
       <c r="AD26" s="7" t="inlineStr">
         <is>
           <t>X</t>
@@ -1868,9 +1898,9 @@
           <t>X</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="17" t="n"/>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="26" t="n"/>
+      <c r="D27" s="27" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
@@ -1891,11 +1921,11 @@
       <c r="V27" s="8" t="n"/>
       <c r="W27" s="8" t="n"/>
       <c r="X27" s="8" t="n"/>
-      <c r="Y27" s="18" t="n"/>
-      <c r="Z27" s="19" t="n"/>
-      <c r="AA27" s="19" t="n"/>
-      <c r="AB27" s="19" t="n"/>
-      <c r="AC27" s="20" t="n"/>
+      <c r="Y27" s="25" t="n"/>
+      <c r="Z27" s="26" t="n"/>
+      <c r="AA27" s="26" t="n"/>
+      <c r="AB27" s="26" t="n"/>
+      <c r="AC27" s="27" t="n"/>
       <c r="AD27" s="7" t="inlineStr">
         <is>
           <t>X</t>
@@ -2073,78 +2103,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>מחלקה</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>אזור</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>מה נמכר כאן</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>דוגמה: מוצרי חלב</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>חלב וביצים</t>
+        </is>
+      </c>
+      <c r="C2" s="29" t="inlineStr">
+        <is>
+          <t>חלב, גבינות, יוגורט, שמנת, חמאה, ביצים</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>מק"ט</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>שם המוצר</t>
         </is>
       </c>
-      <c r="C1" s="21" t="inlineStr">
+      <c r="C1" s="28" t="inlineStr">
         <is>
           <t>שמות נוספים</t>
         </is>
       </c>
-      <c r="D1" s="21" t="inlineStr">
+      <c r="D1" s="28" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="E1" s="21" t="inlineStr">
+      <c r="E1" s="28" t="inlineStr">
         <is>
           <t>אזור</t>
         </is>
       </c>
-      <c r="F1" s="21" t="inlineStr">
+      <c r="F1" s="28" t="inlineStr">
         <is>
           <t>לאסוף בסוף</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>דוגמה: חלב 3%</t>
+          <t>דוגמה: סוללות</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>חלב|חלב בקרטון</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>מוצרי חלב</t>
-        </is>
-      </c>
+          <t>סוללה|סוללות AA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>חלב וביצים</t>
-        </is>
-      </c>
+          <t>קופות</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F3000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"כן"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>